<commit_message>
chore: snapshot legacy budgeting workspace
</commit_message>
<xml_diff>
--- a/base/pacotes/placon-arminio-tavares/parametrico-placon-arminio-tavares.xlsx
+++ b/base/pacotes/placon-arminio-tavares/parametrico-placon-arminio-tavares.xlsx
@@ -42,7 +42,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -132,8 +132,26 @@
       <name val="Arial"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <strike val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -156,6 +174,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F5E9"/>
         <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
+        <bgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -185,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,6 +243,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="17" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3791,7 +3820,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -3801,7 +3830,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -7584,6 +7613,11 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="31" t="inlineStr">
+        <is>
+          <t>OVERRIDES Leo 23/04 (cenário MODERADO): Projetos 500k, Consultorias 150k, Taxas 280k, Almoxarife 3k/mês, Limpeza 75k, EPCs 110k, OpIn 40k, InstProv 110k, DespCons 8,5k/mês. Ger-alvo: R$ 3.089k (17,3%, R$ 758/m²).</t>
+        </is>
+      </c>
       <c r="G2" s="24">
         <f>F24</f>
         <v/>
@@ -7645,8 +7679,8 @@
           <t>vb</t>
         </is>
       </c>
-      <c r="E4" s="26" t="n">
-        <v>650000</v>
+      <c r="E4" s="32" t="n">
+        <v>500000</v>
       </c>
       <c r="F4" s="4">
         <f>C4*E4</f>
@@ -7677,8 +7711,8 @@
           <t>vb</t>
         </is>
       </c>
-      <c r="E5" s="26" t="n">
-        <v>180000</v>
+      <c r="E5" s="32" t="n">
+        <v>150000</v>
       </c>
       <c r="F5" s="4">
         <f>C5*E5</f>
@@ -7741,8 +7775,8 @@
           <t>vb</t>
         </is>
       </c>
-      <c r="E7" s="26" t="n">
-        <v>380000</v>
+      <c r="E7" s="32" t="n">
+        <v>280000</v>
       </c>
       <c r="F7" s="4">
         <f>C7*E7</f>
@@ -7807,8 +7841,8 @@
           <t>mês</t>
         </is>
       </c>
-      <c r="E9" s="26" t="n">
-        <v>9940</v>
+      <c r="E9" s="32" t="n">
+        <v>8000</v>
       </c>
       <c r="F9" s="4">
         <f>C9*E9</f>
@@ -7840,8 +7874,8 @@
           <t>mês</t>
         </is>
       </c>
-      <c r="E10" s="26" t="n">
-        <v>8000</v>
+      <c r="E10" s="32" t="n">
+        <v>6000</v>
       </c>
       <c r="F10" s="4">
         <f>C10*E10</f>
@@ -7854,66 +7888,66 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="33" t="inlineStr">
         <is>
           <t>2×prazo</t>
         </is>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="34">
         <f>DADOS_PROJETO!B11*2</f>
         <v/>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="33" t="inlineStr">
         <is>
           <t>mês</t>
         </is>
       </c>
-      <c r="E11" s="26" t="n">
-        <v>1580</v>
-      </c>
-      <c r="F11" s="4">
+      <c r="E11" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="34">
         <f>C11*E11</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="inlineStr">
+      <c r="G11" s="33" t="inlineStr">
         <is>
           <t>Master R$ 1,6k (3p)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Téc.segurança</t>
         </is>
       </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>1×prazo</t>
         </is>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="34">
         <f>DADOS_PROJETO!B11</f>
         <v/>
       </c>
-      <c r="D12" s="25" t="inlineStr">
+      <c r="D12" s="33" t="inlineStr">
         <is>
           <t>mês</t>
         </is>
       </c>
-      <c r="E12" s="26" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F12" s="4">
+      <c r="E12" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="34">
         <f>C12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="27" t="inlineStr">
+      <c r="G12" s="33" t="inlineStr">
         <is>
           <t>PJ R$ 6k/mês</t>
         </is>
@@ -7939,8 +7973,8 @@
           <t>mês</t>
         </is>
       </c>
-      <c r="E13" s="26" t="n">
-        <v>3377</v>
+      <c r="E13" s="32" t="n">
+        <v>3000</v>
       </c>
       <c r="F13" s="4">
         <f>C13*E13</f>
@@ -7960,20 +7994,19 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>2×prazo</t>
-        </is>
-      </c>
-      <c r="C14" s="4">
-        <f>DADOS_PROJETO!B11*2</f>
-        <v/>
+          <t>1×24m + reforço 6m</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
           <t>mês</t>
         </is>
       </c>
-      <c r="E14" s="26" t="n">
-        <v>2500</v>
+      <c r="E14" s="32" t="n">
+        <v>3125</v>
       </c>
       <c r="F14" s="4">
         <f>C14*E14</f>
@@ -8005,8 +8038,8 @@
           <t>mês</t>
         </is>
       </c>
-      <c r="E15" s="26" t="n">
-        <v>15261</v>
+      <c r="E15" s="32" t="n">
+        <v>5000</v>
       </c>
       <c r="F15" s="4">
         <f>C15*E15</f>
@@ -8037,9 +8070,8 @@
           <t>vb</t>
         </is>
       </c>
-      <c r="E16" s="5">
-        <f>IF(DADOS_PROJETO!B5&lt;5000,150000,IF(DADOS_PROJETO!B5&lt;15000,300000,500000))</f>
-        <v/>
+      <c r="E16" s="32" t="n">
+        <v>110000</v>
       </c>
       <c r="F16" s="4">
         <f>C16*E16</f>
@@ -8135,8 +8167,8 @@
           <t>vb</t>
         </is>
       </c>
-      <c r="E19" s="26" t="n">
-        <v>55000</v>
+      <c r="E19" s="32" t="n">
+        <v>40000</v>
       </c>
       <c r="F19" s="4">
         <f>C19*E19</f>
@@ -8167,8 +8199,8 @@
           <t>vb</t>
         </is>
       </c>
-      <c r="E20" s="26" t="n">
-        <v>160000</v>
+      <c r="E20" s="32" t="n">
+        <v>110000</v>
       </c>
       <c r="F20" s="4">
         <f>C20*E20</f>
@@ -8200,8 +8232,8 @@
           <t>mês</t>
         </is>
       </c>
-      <c r="E21" s="26" t="n">
-        <v>11500</v>
+      <c r="E21" s="32" t="n">
+        <v>8500</v>
       </c>
       <c r="F21" s="4">
         <f>C21*E21</f>

</xml_diff>